<commit_message>
chore: master_data.xlsx 업데이트 (PO매핑 2310→2311행)
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/barcode/master_data.xlsx
+++ b/data/barcode/master_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bjhda\OneDrive\바탕 화면\barcode_server\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BA553A4E-DCB4-401B-9A9F-840AB914AF1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB04EDE4-EDAE-497B-A96F-0AB72344FEA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14400" yWindow="0" windowWidth="14400" windowHeight="15600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PO매핑" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7318" uniqueCount="4677">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7320" uniqueCount="4678">
   <si>
     <t>바코드</t>
   </si>
@@ -14114,6 +14114,10 @@
   </si>
   <si>
     <t>USB-PCI243</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>NNO-콘넥터098</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -14124,7 +14128,7 @@
   <numFmts count="1">
     <numFmt numFmtId="176" formatCode="0_);[Red]\(0\)"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -14151,6 +14155,12 @@
       <color indexed="8"/>
       <name val="NanumGothic"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color indexed="8"/>
+      <name val="나눔고딕"/>
+      <charset val="129"/>
     </font>
   </fonts>
   <fills count="2">
@@ -14188,7 +14198,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -14204,6 +14214,9 @@
     <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="176" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -14510,7 +14523,7 @@
   <dimension ref="A1:B2321"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="16.375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="16.125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10.5" customWidth="1"/>
   </cols>
@@ -33003,8 +33016,13 @@
         <v>4654</v>
       </c>
     </row>
-    <row r="2312" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A2312" s="4"/>
+    <row r="2312" spans="1:2" ht="30" x14ac:dyDescent="0.3">
+      <c r="A2312" s="6" t="s">
+        <v>4412</v>
+      </c>
+      <c r="B2312" t="s">
+        <v>4677</v>
+      </c>
     </row>
     <row r="2313" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2313" s="4"/>

</xml_diff>